<commit_message>
full replace app with contact master editing
</commit_message>
<xml_diff>
--- a/quotation_template.xlsx
+++ b/quotation_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kenseikobayashi/Desktop/report_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D26D8D2B-50ED-374F-A97E-E0C7E6C6B85C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EDDF5BA-39CE-FA4F-B508-C5EBBDC3DF9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7980" yWindow="660" windowWidth="29400" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="見積書" sheetId="1" r:id="rId1"/>
@@ -250,24 +250,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="9"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <name val="Arial (本文)"/>
+      <family val="3"/>
       <charset val="128"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <sz val="9"/>
+      <name val="Arial (本文)"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="9"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Arial (本文)"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="5">
@@ -466,7 +466,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -502,6 +502,11 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -513,9 +518,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -552,6 +555,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -808,26 +814,26 @@
       <c r="J3" s="4"/>
     </row>
     <row r="4" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="35"/>
-      <c r="J4" s="35"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="38"/>
+      <c r="J4" s="38"/>
     </row>
     <row r="5" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="H5" s="5"/>
     </row>
     <row r="6" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="36"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
+      <c r="B6" s="39"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
       <c r="E6" s="6" t="s">
         <v>4</v>
       </c>
@@ -883,37 +889,37 @@
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="40">
+      <c r="C15" s="43">
         <f>I28</f>
         <v>0</v>
       </c>
-      <c r="D15" s="41"/>
-      <c r="E15" s="43" t="s">
+      <c r="D15" s="44"/>
+      <c r="E15" s="46" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B16" s="39"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="44"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="47"/>
     </row>
     <row r="17" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="18" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="9"/>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="32" t="s">
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="30"/>
+      <c r="G18" s="33"/>
       <c r="H18" s="10" t="s">
         <v>18</v>
       </c>
@@ -922,106 +928,106 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="28"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13">
+      <c r="B19" s="31"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="21">
         <f t="shared" ref="I19:I20" si="0">F19*H19</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="28"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="13">
+      <c r="B20" s="31"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="21">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="28"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="14"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="21"/>
+      <c r="I21" s="20"/>
     </row>
     <row r="22" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="28"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="14"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="20"/>
     </row>
     <row r="23" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="28"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="14"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="20"/>
     </row>
     <row r="24" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="28"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="14"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="20"/>
     </row>
     <row r="25" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="28"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="14"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="20"/>
     </row>
     <row r="26" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="28"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="14"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="33"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="20"/>
     </row>
     <row r="27" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="28"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="11"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="14"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="20"/>
     </row>
     <row r="28" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="H28" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="I28" s="13">
+      <c r="I28" s="21">
         <f>SUM(I19:I27)</f>
         <v>0</v>
       </c>
@@ -1030,7 +1036,7 @@
       <c r="H29" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="I29" s="13">
+      <c r="I29" s="21">
         <f>I28*0.1</f>
         <v>0</v>
       </c>
@@ -1039,7 +1045,7 @@
       <c r="H30" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="I30" s="13">
+      <c r="I30" s="21">
         <f>I28+I29</f>
         <v>0</v>
       </c>
@@ -1055,146 +1061,146 @@
       <c r="I31" s="16"/>
     </row>
     <row r="32" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="33" t="s">
+      <c r="B32" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="30"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="33"/>
     </row>
     <row r="33" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B33" s="19"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
-      <c r="I33" s="21"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="24"/>
     </row>
     <row r="34" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B34" s="22"/>
-      <c r="C34" s="23"/>
-      <c r="D34" s="23"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="23"/>
-      <c r="I34" s="24"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="27"/>
     </row>
     <row r="35" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B35" s="22"/>
-      <c r="C35" s="23"/>
-      <c r="D35" s="23"/>
-      <c r="E35" s="23"/>
-      <c r="F35" s="23"/>
-      <c r="G35" s="23"/>
-      <c r="H35" s="23"/>
-      <c r="I35" s="24"/>
+      <c r="B35" s="25"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="26"/>
+      <c r="G35" s="26"/>
+      <c r="H35" s="26"/>
+      <c r="I35" s="27"/>
     </row>
     <row r="36" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B36" s="22"/>
-      <c r="C36" s="23"/>
-      <c r="D36" s="23"/>
-      <c r="E36" s="23"/>
-      <c r="F36" s="23"/>
-      <c r="G36" s="23"/>
-      <c r="H36" s="23"/>
-      <c r="I36" s="24"/>
+      <c r="B36" s="25"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="26"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="27"/>
     </row>
     <row r="37" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B37" s="22"/>
-      <c r="C37" s="23"/>
-      <c r="D37" s="23"/>
-      <c r="E37" s="23"/>
-      <c r="F37" s="23"/>
-      <c r="G37" s="23"/>
-      <c r="H37" s="23"/>
-      <c r="I37" s="24"/>
+      <c r="B37" s="25"/>
+      <c r="C37" s="26"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="26"/>
+      <c r="F37" s="26"/>
+      <c r="G37" s="26"/>
+      <c r="H37" s="26"/>
+      <c r="I37" s="27"/>
     </row>
     <row r="38" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B38" s="22"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="23"/>
-      <c r="F38" s="23"/>
-      <c r="G38" s="23"/>
-      <c r="H38" s="23"/>
-      <c r="I38" s="24"/>
+      <c r="B38" s="25"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="26"/>
+      <c r="F38" s="26"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="26"/>
+      <c r="I38" s="27"/>
     </row>
     <row r="39" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B39" s="22"/>
-      <c r="C39" s="23"/>
-      <c r="D39" s="23"/>
-      <c r="E39" s="23"/>
-      <c r="F39" s="23"/>
-      <c r="G39" s="23"/>
-      <c r="H39" s="23"/>
-      <c r="I39" s="24"/>
+      <c r="B39" s="25"/>
+      <c r="C39" s="26"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="26"/>
+      <c r="F39" s="26"/>
+      <c r="G39" s="26"/>
+      <c r="H39" s="26"/>
+      <c r="I39" s="27"/>
     </row>
     <row r="40" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B40" s="22"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
-      <c r="H40" s="23"/>
-      <c r="I40" s="24"/>
+      <c r="B40" s="25"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="26"/>
+      <c r="F40" s="26"/>
+      <c r="G40" s="26"/>
+      <c r="H40" s="26"/>
+      <c r="I40" s="27"/>
     </row>
     <row r="41" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B41" s="22"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="23"/>
-      <c r="E41" s="23"/>
-      <c r="F41" s="23"/>
-      <c r="G41" s="23"/>
-      <c r="H41" s="23"/>
-      <c r="I41" s="24"/>
+      <c r="B41" s="25"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="26"/>
+      <c r="F41" s="26"/>
+      <c r="G41" s="26"/>
+      <c r="H41" s="26"/>
+      <c r="I41" s="27"/>
     </row>
     <row r="42" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B42" s="22"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="23"/>
-      <c r="E42" s="23"/>
-      <c r="F42" s="23"/>
-      <c r="G42" s="23"/>
-      <c r="H42" s="23"/>
-      <c r="I42" s="24"/>
+      <c r="B42" s="25"/>
+      <c r="C42" s="26"/>
+      <c r="D42" s="26"/>
+      <c r="E42" s="26"/>
+      <c r="F42" s="26"/>
+      <c r="G42" s="26"/>
+      <c r="H42" s="26"/>
+      <c r="I42" s="27"/>
     </row>
     <row r="43" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="B43" s="22"/>
-      <c r="C43" s="23"/>
-      <c r="D43" s="23"/>
-      <c r="E43" s="23"/>
-      <c r="F43" s="23"/>
-      <c r="G43" s="23"/>
-      <c r="H43" s="23"/>
-      <c r="I43" s="24"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="26"/>
+      <c r="D43" s="26"/>
+      <c r="E43" s="26"/>
+      <c r="F43" s="26"/>
+      <c r="G43" s="26"/>
+      <c r="H43" s="26"/>
+      <c r="I43" s="27"/>
     </row>
     <row r="44" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="B44" s="22"/>
-      <c r="C44" s="23"/>
-      <c r="D44" s="23"/>
-      <c r="E44" s="23"/>
-      <c r="F44" s="23"/>
-      <c r="G44" s="23"/>
-      <c r="H44" s="23"/>
-      <c r="I44" s="24"/>
+      <c r="B44" s="25"/>
+      <c r="C44" s="26"/>
+      <c r="D44" s="26"/>
+      <c r="E44" s="26"/>
+      <c r="F44" s="26"/>
+      <c r="G44" s="26"/>
+      <c r="H44" s="26"/>
+      <c r="I44" s="27"/>
     </row>
     <row r="45" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="B45" s="25"/>
-      <c r="C45" s="26"/>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="26"/>
-      <c r="I45" s="27"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="29"/>
+      <c r="D45" s="29"/>
+      <c r="E45" s="29"/>
+      <c r="F45" s="29"/>
+      <c r="G45" s="29"/>
+      <c r="H45" s="29"/>
+      <c r="I45" s="30"/>
     </row>
     <row r="46" spans="2:9" ht="13" x14ac:dyDescent="0.15">
       <c r="B46" s="17"/>
@@ -1289,28 +1295,28 @@
       <c r="J3" s="4"/>
     </row>
     <row r="4" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="35"/>
-      <c r="J4" s="35"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="38"/>
+      <c r="J4" s="38"/>
     </row>
     <row r="5" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="H5" s="5"/>
     </row>
     <row r="6" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
       <c r="E6" s="6" t="s">
         <v>4</v>
       </c>
@@ -1377,37 +1383,37 @@
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="40">
+      <c r="C15" s="43">
         <f>I28</f>
         <v>1998000</v>
       </c>
-      <c r="D15" s="41"/>
-      <c r="E15" s="43" t="s">
+      <c r="D15" s="44"/>
+      <c r="E15" s="46" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B16" s="39"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="44"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="47"/>
     </row>
     <row r="17" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="18" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="9"/>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="32" t="s">
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="30"/>
+      <c r="G18" s="33"/>
       <c r="H18" s="10" t="s">
         <v>18</v>
       </c>
@@ -1416,12 +1422,12 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="30"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="33"/>
       <c r="F19" s="11">
         <v>1</v>
       </c>
@@ -1437,12 +1443,12 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="30"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="33"/>
       <c r="F20" s="11">
         <v>1</v>
       </c>
@@ -1458,70 +1464,70 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="28"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="30"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="33"/>
       <c r="F21" s="11"/>
       <c r="G21" s="12"/>
       <c r="H21" s="13"/>
       <c r="I21" s="14"/>
     </row>
     <row r="22" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="28"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="30"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="33"/>
       <c r="F22" s="11"/>
       <c r="G22" s="12"/>
       <c r="H22" s="13"/>
       <c r="I22" s="14"/>
     </row>
     <row r="23" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="28"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="30"/>
+      <c r="B23" s="52"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="33"/>
       <c r="F23" s="11"/>
       <c r="G23" s="12"/>
       <c r="H23" s="13"/>
       <c r="I23" s="14"/>
     </row>
     <row r="24" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="28"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="30"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="33"/>
       <c r="F24" s="11"/>
       <c r="G24" s="12"/>
       <c r="H24" s="13"/>
       <c r="I24" s="14"/>
     </row>
     <row r="25" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="28"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="30"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="11"/>
       <c r="G25" s="12"/>
       <c r="H25" s="13"/>
       <c r="I25" s="14"/>
     </row>
     <row r="26" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="28"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="30"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="33"/>
       <c r="F26" s="11"/>
       <c r="G26" s="12"/>
       <c r="H26" s="13"/>
       <c r="I26" s="14"/>
     </row>
     <row r="27" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="28"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="30"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="33"/>
       <c r="F27" s="11"/>
       <c r="G27" s="12"/>
       <c r="H27" s="13"/>
@@ -1565,148 +1571,148 @@
       <c r="I31" s="16"/>
     </row>
     <row r="32" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="33" t="s">
+      <c r="B32" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="30"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="33"/>
     </row>
     <row r="33" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B33" s="45" t="s">
+      <c r="B33" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="46"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="44"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="44"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="49"/>
     </row>
     <row r="34" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B34" s="47"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
-      <c r="G34" s="35"/>
-      <c r="H34" s="35"/>
-      <c r="I34" s="48"/>
+      <c r="B34" s="50"/>
+      <c r="C34" s="38"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="51"/>
     </row>
     <row r="35" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B35" s="47"/>
-      <c r="C35" s="35"/>
-      <c r="D35" s="35"/>
-      <c r="E35" s="35"/>
-      <c r="F35" s="35"/>
-      <c r="G35" s="35"/>
-      <c r="H35" s="35"/>
-      <c r="I35" s="48"/>
+      <c r="B35" s="50"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="51"/>
     </row>
     <row r="36" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B36" s="47"/>
-      <c r="C36" s="35"/>
-      <c r="D36" s="35"/>
-      <c r="E36" s="35"/>
-      <c r="F36" s="35"/>
-      <c r="G36" s="35"/>
-      <c r="H36" s="35"/>
-      <c r="I36" s="48"/>
+      <c r="B36" s="50"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="51"/>
     </row>
     <row r="37" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B37" s="47"/>
-      <c r="C37" s="35"/>
-      <c r="D37" s="35"/>
-      <c r="E37" s="35"/>
-      <c r="F37" s="35"/>
-      <c r="G37" s="35"/>
-      <c r="H37" s="35"/>
-      <c r="I37" s="48"/>
+      <c r="B37" s="50"/>
+      <c r="C37" s="38"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="38"/>
+      <c r="I37" s="51"/>
     </row>
     <row r="38" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B38" s="47"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="35"/>
-      <c r="F38" s="35"/>
-      <c r="G38" s="35"/>
-      <c r="H38" s="35"/>
-      <c r="I38" s="48"/>
+      <c r="B38" s="50"/>
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="51"/>
     </row>
     <row r="39" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B39" s="47"/>
-      <c r="C39" s="35"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="35"/>
-      <c r="F39" s="35"/>
-      <c r="G39" s="35"/>
-      <c r="H39" s="35"/>
-      <c r="I39" s="48"/>
+      <c r="B39" s="50"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="38"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="51"/>
     </row>
     <row r="40" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B40" s="47"/>
-      <c r="C40" s="35"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35"/>
-      <c r="F40" s="35"/>
-      <c r="G40" s="35"/>
-      <c r="H40" s="35"/>
-      <c r="I40" s="48"/>
+      <c r="B40" s="50"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="38"/>
+      <c r="G40" s="38"/>
+      <c r="H40" s="38"/>
+      <c r="I40" s="51"/>
     </row>
     <row r="41" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B41" s="47"/>
-      <c r="C41" s="35"/>
-      <c r="D41" s="35"/>
-      <c r="E41" s="35"/>
-      <c r="F41" s="35"/>
-      <c r="G41" s="35"/>
-      <c r="H41" s="35"/>
-      <c r="I41" s="48"/>
+      <c r="B41" s="50"/>
+      <c r="C41" s="38"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="38"/>
+      <c r="F41" s="38"/>
+      <c r="G41" s="38"/>
+      <c r="H41" s="38"/>
+      <c r="I41" s="51"/>
     </row>
     <row r="42" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B42" s="47"/>
-      <c r="C42" s="35"/>
-      <c r="D42" s="35"/>
-      <c r="E42" s="35"/>
-      <c r="F42" s="35"/>
-      <c r="G42" s="35"/>
-      <c r="H42" s="35"/>
-      <c r="I42" s="48"/>
+      <c r="B42" s="50"/>
+      <c r="C42" s="38"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="38"/>
+      <c r="G42" s="38"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="51"/>
     </row>
     <row r="43" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="B43" s="47"/>
-      <c r="C43" s="35"/>
-      <c r="D43" s="35"/>
-      <c r="E43" s="35"/>
-      <c r="F43" s="35"/>
-      <c r="G43" s="35"/>
-      <c r="H43" s="35"/>
-      <c r="I43" s="48"/>
+      <c r="B43" s="50"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="38"/>
+      <c r="H43" s="38"/>
+      <c r="I43" s="51"/>
     </row>
     <row r="44" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="B44" s="47"/>
-      <c r="C44" s="35"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="35"/>
-      <c r="F44" s="35"/>
-      <c r="G44" s="35"/>
-      <c r="H44" s="35"/>
-      <c r="I44" s="48"/>
+      <c r="B44" s="50"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38"/>
+      <c r="G44" s="38"/>
+      <c r="H44" s="38"/>
+      <c r="I44" s="51"/>
     </row>
     <row r="45" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="B45" s="42"/>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="37"/>
-      <c r="F45" s="37"/>
-      <c r="G45" s="37"/>
-      <c r="H45" s="37"/>
-      <c r="I45" s="44"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="40"/>
+      <c r="E45" s="40"/>
+      <c r="F45" s="40"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="40"/>
+      <c r="I45" s="47"/>
     </row>
     <row r="46" spans="2:9" ht="13" x14ac:dyDescent="0.15">
       <c r="B46" s="17"/>
@@ -1801,28 +1807,28 @@
       <c r="J3" s="4"/>
     </row>
     <row r="4" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="35"/>
-      <c r="J4" s="35"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="38"/>
+      <c r="J4" s="38"/>
     </row>
     <row r="5" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="H5" s="5"/>
     </row>
     <row r="6" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
       <c r="E6" s="6" t="s">
         <v>4</v>
       </c>
@@ -1889,37 +1895,37 @@
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="40">
+      <c r="C15" s="43">
         <f>I28</f>
         <v>1998000</v>
       </c>
-      <c r="D15" s="41"/>
-      <c r="E15" s="43" t="s">
+      <c r="D15" s="44"/>
+      <c r="E15" s="46" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B16" s="39"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="44"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="47"/>
     </row>
     <row r="17" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="18" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="9"/>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="32" t="s">
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="30"/>
+      <c r="G18" s="33"/>
       <c r="H18" s="10" t="s">
         <v>18</v>
       </c>
@@ -1928,12 +1934,12 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="30"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="33"/>
       <c r="F19" s="11">
         <v>1</v>
       </c>
@@ -1949,12 +1955,12 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="30"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="33"/>
       <c r="F20" s="11">
         <v>1</v>
       </c>
@@ -1970,70 +1976,70 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="28"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="30"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="33"/>
       <c r="F21" s="11"/>
       <c r="G21" s="12"/>
       <c r="H21" s="13"/>
       <c r="I21" s="14"/>
     </row>
     <row r="22" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="28"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="30"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="33"/>
       <c r="F22" s="11"/>
       <c r="G22" s="12"/>
       <c r="H22" s="13"/>
       <c r="I22" s="14"/>
     </row>
     <row r="23" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="28"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="30"/>
+      <c r="B23" s="52"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="33"/>
       <c r="F23" s="11"/>
       <c r="G23" s="12"/>
       <c r="H23" s="13"/>
       <c r="I23" s="14"/>
     </row>
     <row r="24" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="28"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="30"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="33"/>
       <c r="F24" s="11"/>
       <c r="G24" s="12"/>
       <c r="H24" s="13"/>
       <c r="I24" s="14"/>
     </row>
     <row r="25" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="28"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="30"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="11"/>
       <c r="G25" s="12"/>
       <c r="H25" s="13"/>
       <c r="I25" s="14"/>
     </row>
     <row r="26" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="28"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="30"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="33"/>
       <c r="F26" s="11"/>
       <c r="G26" s="12"/>
       <c r="H26" s="13"/>
       <c r="I26" s="14"/>
     </row>
     <row r="27" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="28"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="30"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="33"/>
       <c r="F27" s="11"/>
       <c r="G27" s="12"/>
       <c r="H27" s="13"/>
@@ -2077,148 +2083,148 @@
       <c r="I31" s="16"/>
     </row>
     <row r="32" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="33" t="s">
+      <c r="B32" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="29"/>
-      <c r="H32" s="29"/>
-      <c r="I32" s="30"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="33"/>
     </row>
     <row r="33" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B33" s="45" t="s">
+      <c r="B33" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="C33" s="41"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="46"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="44"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="44"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="49"/>
     </row>
     <row r="34" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B34" s="47"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
-      <c r="G34" s="35"/>
-      <c r="H34" s="35"/>
-      <c r="I34" s="48"/>
+      <c r="B34" s="50"/>
+      <c r="C34" s="38"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="51"/>
     </row>
     <row r="35" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B35" s="47"/>
-      <c r="C35" s="35"/>
-      <c r="D35" s="35"/>
-      <c r="E35" s="35"/>
-      <c r="F35" s="35"/>
-      <c r="G35" s="35"/>
-      <c r="H35" s="35"/>
-      <c r="I35" s="48"/>
+      <c r="B35" s="50"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="51"/>
     </row>
     <row r="36" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B36" s="47"/>
-      <c r="C36" s="35"/>
-      <c r="D36" s="35"/>
-      <c r="E36" s="35"/>
-      <c r="F36" s="35"/>
-      <c r="G36" s="35"/>
-      <c r="H36" s="35"/>
-      <c r="I36" s="48"/>
+      <c r="B36" s="50"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="51"/>
     </row>
     <row r="37" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B37" s="47"/>
-      <c r="C37" s="35"/>
-      <c r="D37" s="35"/>
-      <c r="E37" s="35"/>
-      <c r="F37" s="35"/>
-      <c r="G37" s="35"/>
-      <c r="H37" s="35"/>
-      <c r="I37" s="48"/>
+      <c r="B37" s="50"/>
+      <c r="C37" s="38"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="38"/>
+      <c r="I37" s="51"/>
     </row>
     <row r="38" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B38" s="47"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="35"/>
-      <c r="F38" s="35"/>
-      <c r="G38" s="35"/>
-      <c r="H38" s="35"/>
-      <c r="I38" s="48"/>
+      <c r="B38" s="50"/>
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="51"/>
     </row>
     <row r="39" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B39" s="47"/>
-      <c r="C39" s="35"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="35"/>
-      <c r="F39" s="35"/>
-      <c r="G39" s="35"/>
-      <c r="H39" s="35"/>
-      <c r="I39" s="48"/>
+      <c r="B39" s="50"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="38"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="51"/>
     </row>
     <row r="40" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B40" s="47"/>
-      <c r="C40" s="35"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35"/>
-      <c r="F40" s="35"/>
-      <c r="G40" s="35"/>
-      <c r="H40" s="35"/>
-      <c r="I40" s="48"/>
+      <c r="B40" s="50"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="38"/>
+      <c r="G40" s="38"/>
+      <c r="H40" s="38"/>
+      <c r="I40" s="51"/>
     </row>
     <row r="41" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B41" s="47"/>
-      <c r="C41" s="35"/>
-      <c r="D41" s="35"/>
-      <c r="E41" s="35"/>
-      <c r="F41" s="35"/>
-      <c r="G41" s="35"/>
-      <c r="H41" s="35"/>
-      <c r="I41" s="48"/>
+      <c r="B41" s="50"/>
+      <c r="C41" s="38"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="38"/>
+      <c r="F41" s="38"/>
+      <c r="G41" s="38"/>
+      <c r="H41" s="38"/>
+      <c r="I41" s="51"/>
     </row>
     <row r="42" spans="2:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B42" s="47"/>
-      <c r="C42" s="35"/>
-      <c r="D42" s="35"/>
-      <c r="E42" s="35"/>
-      <c r="F42" s="35"/>
-      <c r="G42" s="35"/>
-      <c r="H42" s="35"/>
-      <c r="I42" s="48"/>
+      <c r="B42" s="50"/>
+      <c r="C42" s="38"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="38"/>
+      <c r="G42" s="38"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="51"/>
     </row>
     <row r="43" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="B43" s="47"/>
-      <c r="C43" s="35"/>
-      <c r="D43" s="35"/>
-      <c r="E43" s="35"/>
-      <c r="F43" s="35"/>
-      <c r="G43" s="35"/>
-      <c r="H43" s="35"/>
-      <c r="I43" s="48"/>
+      <c r="B43" s="50"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="38"/>
+      <c r="H43" s="38"/>
+      <c r="I43" s="51"/>
     </row>
     <row r="44" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="B44" s="47"/>
-      <c r="C44" s="35"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="35"/>
-      <c r="F44" s="35"/>
-      <c r="G44" s="35"/>
-      <c r="H44" s="35"/>
-      <c r="I44" s="48"/>
+      <c r="B44" s="50"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38"/>
+      <c r="G44" s="38"/>
+      <c r="H44" s="38"/>
+      <c r="I44" s="51"/>
     </row>
     <row r="45" spans="2:9" ht="13" x14ac:dyDescent="0.15">
-      <c r="B45" s="42"/>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="37"/>
-      <c r="F45" s="37"/>
-      <c r="G45" s="37"/>
-      <c r="H45" s="37"/>
-      <c r="I45" s="44"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="40"/>
+      <c r="E45" s="40"/>
+      <c r="F45" s="40"/>
+      <c r="G45" s="40"/>
+      <c r="H45" s="40"/>
+      <c r="I45" s="47"/>
     </row>
     <row r="46" spans="2:9" ht="13" x14ac:dyDescent="0.15">
       <c r="B46" s="17"/>

</xml_diff>